<commit_message>
ajuste y limpieza de metodos
se grafica comportamiento de pureza por entropia
</commit_message>
<xml_diff>
--- a/codigo/datasets/datasets_aumentados/logs/pcsmote/por_muestras/log_pcsmote_x_muestra_ecoli.xlsx
+++ b/codigo/datasets/datasets_aumentados/logs/pcsmote/por_muestras/log_pcsmote_x_muestra_ecoli.xlsx
@@ -621,7 +621,7 @@
         <v>7</v>
       </c>
       <c r="U2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V2">
         <v>7</v>
@@ -692,7 +692,7 @@
         <v>7</v>
       </c>
       <c r="U3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="V3">
         <v>7</v>
@@ -899,7 +899,7 @@
         <v>1</v>
       </c>
       <c r="S6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T6">
         <v>7</v>
@@ -1035,13 +1035,13 @@
         <v>0.4285714285714285</v>
       </c>
       <c r="Q8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R8" t="b">
         <v>1</v>
       </c>
       <c r="S8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T8">
         <v>7</v>
@@ -1118,7 +1118,7 @@
         <v>7</v>
       </c>
       <c r="U9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V9">
         <v>7</v>
@@ -1473,7 +1473,7 @@
         <v>7</v>
       </c>
       <c r="U14">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="V14">
         <v>7</v>
@@ -1609,7 +1609,7 @@
         <v>1</v>
       </c>
       <c r="S16" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T16">
         <v>7</v>
@@ -1893,7 +1893,7 @@
         <v>1</v>
       </c>
       <c r="S20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T20">
         <v>7</v>
@@ -2112,7 +2112,7 @@
         <v>7</v>
       </c>
       <c r="U23">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V23">
         <v>7</v>
@@ -2248,7 +2248,7 @@
         <v>1</v>
       </c>
       <c r="S25" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T25">
         <v>7</v>
@@ -2325,7 +2325,7 @@
         <v>7</v>
       </c>
       <c r="U26">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="V26">
         <v>7</v>
@@ -2396,7 +2396,7 @@
         <v>7</v>
       </c>
       <c r="U27">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V27">
         <v>7</v>
@@ -2467,7 +2467,7 @@
         <v>7</v>
       </c>
       <c r="U28">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V28">
         <v>7</v>
@@ -2538,7 +2538,7 @@
         <v>7</v>
       </c>
       <c r="U29">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V29">
         <v>7</v>
@@ -2603,7 +2603,7 @@
         <v>1</v>
       </c>
       <c r="S30" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T30">
         <v>7</v>
@@ -2680,7 +2680,7 @@
         <v>7</v>
       </c>
       <c r="U31">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V31">
         <v>7</v>
@@ -2751,7 +2751,7 @@
         <v>7</v>
       </c>
       <c r="U32">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V32">
         <v>7</v>
@@ -2822,7 +2822,7 @@
         <v>7</v>
       </c>
       <c r="U33">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V33">
         <v>7</v>
@@ -2893,7 +2893,7 @@
         <v>7</v>
       </c>
       <c r="U34">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V34">
         <v>7</v>
@@ -2964,7 +2964,7 @@
         <v>7</v>
       </c>
       <c r="U35">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V35">
         <v>7</v>
@@ -3023,7 +3023,7 @@
         <v>0</v>
       </c>
       <c r="Q36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R36" t="b">
         <v>0</v>
@@ -3836,7 +3836,7 @@
         <v>25</v>
       </c>
       <c r="D48" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E48">
         <v>7</v>
@@ -3878,7 +3878,7 @@
         <v>1</v>
       </c>
       <c r="R48" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S48" t="b">
         <v>1</v>
@@ -3887,7 +3887,7 @@
         <v>6</v>
       </c>
       <c r="U48">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="V48">
         <v>6</v>
@@ -3978,7 +3978,7 @@
         <v>25</v>
       </c>
       <c r="D50" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E50">
         <v>7</v>
@@ -4020,7 +4020,7 @@
         <v>1</v>
       </c>
       <c r="R50" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S50" t="b">
         <v>1</v>
@@ -4372,7 +4372,7 @@
         <v>0.7142857142857143</v>
       </c>
       <c r="Q55" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R55" t="b">
         <v>1</v>
@@ -4455,7 +4455,7 @@
         <v>7</v>
       </c>
       <c r="U56">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="V56">
         <v>7</v>
@@ -4520,7 +4520,7 @@
         <v>1</v>
       </c>
       <c r="S57" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T57">
         <v>7</v>
@@ -4798,7 +4798,7 @@
         <v>0</v>
       </c>
       <c r="Q61" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R61" t="b">
         <v>0</v>
@@ -4881,7 +4881,7 @@
         <v>7</v>
       </c>
       <c r="U62">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V62">
         <v>7</v>
@@ -5230,7 +5230,7 @@
         <v>1</v>
       </c>
       <c r="S67" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T67">
         <v>7</v>
@@ -5301,7 +5301,7 @@
         <v>0</v>
       </c>
       <c r="S68" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T68">
         <v>5</v>
@@ -5327,7 +5327,7 @@
         <v>26</v>
       </c>
       <c r="D69" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E69">
         <v>7</v>
@@ -5366,7 +5366,7 @@
         <v>0</v>
       </c>
       <c r="Q69" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R69" t="b">
         <v>1</v>
@@ -5378,7 +5378,7 @@
         <v>7</v>
       </c>
       <c r="U69">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="V69">
         <v>7</v>
@@ -5656,7 +5656,7 @@
         <v>1</v>
       </c>
       <c r="S73" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T73">
         <v>7</v>
@@ -5875,7 +5875,7 @@
         <v>7</v>
       </c>
       <c r="U76">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="V76">
         <v>7</v>
@@ -5946,7 +5946,7 @@
         <v>7</v>
       </c>
       <c r="U77">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="V77">
         <v>7</v>
@@ -6082,7 +6082,7 @@
         <v>1</v>
       </c>
       <c r="S79" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T79">
         <v>7</v>
@@ -6301,7 +6301,7 @@
         <v>7</v>
       </c>
       <c r="U82">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="V82">
         <v>7</v>
@@ -6437,7 +6437,7 @@
         <v>1</v>
       </c>
       <c r="S84" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T84">
         <v>7</v>
@@ -6579,7 +6579,7 @@
         <v>1</v>
       </c>
       <c r="S86" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T86">
         <v>7</v>
@@ -6715,7 +6715,7 @@
         <v>0.8571428571428571</v>
       </c>
       <c r="Q88" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R88" t="b">
         <v>1</v>
@@ -6798,7 +6798,7 @@
         <v>7</v>
       </c>
       <c r="U89">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="V89">
         <v>7</v>
@@ -6889,7 +6889,7 @@
         <v>27</v>
       </c>
       <c r="D91" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E91">
         <v>7</v>
@@ -6931,7 +6931,7 @@
         <v>1</v>
       </c>
       <c r="R91" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S91" t="b">
         <v>1</v>
@@ -6940,7 +6940,7 @@
         <v>6</v>
       </c>
       <c r="U91">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="V91">
         <v>6</v>
@@ -6960,7 +6960,7 @@
         <v>27</v>
       </c>
       <c r="D92" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E92">
         <v>7</v>
@@ -7002,7 +7002,7 @@
         <v>1</v>
       </c>
       <c r="R92" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S92" t="b">
         <v>1</v>
@@ -7011,7 +7011,7 @@
         <v>7</v>
       </c>
       <c r="U92">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="V92">
         <v>7</v>
@@ -7031,7 +7031,7 @@
         <v>27</v>
       </c>
       <c r="D93" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E93">
         <v>7</v>
@@ -7073,7 +7073,7 @@
         <v>1</v>
       </c>
       <c r="R93" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S93" t="b">
         <v>1</v>
@@ -7082,7 +7082,7 @@
         <v>7</v>
       </c>
       <c r="U93">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="V93">
         <v>7</v>
@@ -7102,7 +7102,7 @@
         <v>27</v>
       </c>
       <c r="D94" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E94">
         <v>7</v>
@@ -7144,7 +7144,7 @@
         <v>1</v>
       </c>
       <c r="R94" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S94" t="b">
         <v>1</v>
@@ -7153,7 +7153,7 @@
         <v>6</v>
       </c>
       <c r="U94">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="V94">
         <v>6</v>
@@ -7215,7 +7215,7 @@
         <v>0</v>
       </c>
       <c r="R95" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S95" t="b">
         <v>0</v>
@@ -7357,10 +7357,10 @@
         <v>0</v>
       </c>
       <c r="R97" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S97" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T97">
         <v>7</v>
@@ -7570,7 +7570,7 @@
         <v>0</v>
       </c>
       <c r="R100" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S100" t="b">
         <v>1</v>
@@ -7712,10 +7712,10 @@
         <v>0</v>
       </c>
       <c r="R102" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S102" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T102">
         <v>7</v>
@@ -7741,7 +7741,7 @@
         <v>27</v>
       </c>
       <c r="D103" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E103">
         <v>7</v>
@@ -7783,7 +7783,7 @@
         <v>1</v>
       </c>
       <c r="R103" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S103" t="b">
         <v>1</v>
@@ -7792,7 +7792,7 @@
         <v>6</v>
       </c>
       <c r="U103">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="V103">
         <v>6</v>
@@ -7851,13 +7851,13 @@
         <v>0.4285714285714285</v>
       </c>
       <c r="Q104" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R104" t="b">
         <v>0</v>
       </c>
       <c r="S104" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T104">
         <v>3</v>
@@ -7925,10 +7925,10 @@
         <v>0</v>
       </c>
       <c r="R105" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S105" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T105">
         <v>7</v>
@@ -8076,7 +8076,7 @@
         <v>7</v>
       </c>
       <c r="U107">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="V107">
         <v>7</v>
@@ -8141,7 +8141,7 @@
         <v>0</v>
       </c>
       <c r="S108" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T108">
         <v>4</v>
@@ -8360,7 +8360,7 @@
         <v>7</v>
       </c>
       <c r="U111">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V111">
         <v>7</v>
@@ -8573,7 +8573,7 @@
         <v>7</v>
       </c>
       <c r="U114">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="V114">
         <v>7</v>
@@ -9277,7 +9277,7 @@
         <v>1</v>
       </c>
       <c r="S124" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T124">
         <v>7</v>
@@ -9638,7 +9638,7 @@
         <v>7</v>
       </c>
       <c r="U129">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="V129">
         <v>7</v>
@@ -9703,7 +9703,7 @@
         <v>1</v>
       </c>
       <c r="S130" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T130">
         <v>7</v>
@@ -9851,7 +9851,7 @@
         <v>7</v>
       </c>
       <c r="U132">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="V132">
         <v>7</v>
@@ -10064,7 +10064,7 @@
         <v>7</v>
       </c>
       <c r="U135">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="V135">
         <v>7</v>
@@ -10129,7 +10129,7 @@
         <v>1</v>
       </c>
       <c r="S136" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T136">
         <v>7</v>
@@ -10206,7 +10206,7 @@
         <v>7</v>
       </c>
       <c r="U137">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="V137">
         <v>7</v>
@@ -10277,7 +10277,7 @@
         <v>6</v>
       </c>
       <c r="U138">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="V138">
         <v>6</v>
@@ -10703,7 +10703,7 @@
         <v>7</v>
       </c>
       <c r="U144">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="V144">
         <v>7</v>
@@ -11046,7 +11046,7 @@
         <v>7</v>
       </c>
       <c r="U149">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="V149">
         <v>7</v>
@@ -11196,7 +11196,7 @@
         <v>25</v>
       </c>
       <c r="D152" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E152">
         <v>7</v>
@@ -11235,13 +11235,13 @@
         <v>1</v>
       </c>
       <c r="S152" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T152">
         <v>7</v>
       </c>
       <c r="U152">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="V152">
         <v>7</v>
@@ -11365,7 +11365,7 @@
         <v>1</v>
       </c>
       <c r="S154" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T154">
         <v>7</v>
@@ -11436,7 +11436,7 @@
         <v>7</v>
       </c>
       <c r="U155">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="V155">
         <v>7</v>
@@ -11631,7 +11631,7 @@
         <v>7</v>
       </c>
       <c r="U158">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="V158">
         <v>7</v>
@@ -11846,7 +11846,7 @@
         <v>25</v>
       </c>
       <c r="D162" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E162">
         <v>7</v>
@@ -11885,13 +11885,13 @@
         <v>1</v>
       </c>
       <c r="S162" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T162">
         <v>7</v>
       </c>
       <c r="U162">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="V162">
         <v>7</v>
@@ -12106,7 +12106,7 @@
         <v>25</v>
       </c>
       <c r="D166" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E166">
         <v>7</v>
@@ -12145,13 +12145,13 @@
         <v>1</v>
       </c>
       <c r="S166" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T166">
         <v>7</v>
       </c>
       <c r="U166">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="V166">
         <v>7</v>
@@ -12346,7 +12346,7 @@
         <v>7</v>
       </c>
       <c r="U169">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="V169">
         <v>7</v>
@@ -12470,7 +12470,7 @@
         <v>1</v>
       </c>
       <c r="S171" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T171">
         <v>7</v>
@@ -12606,7 +12606,7 @@
         <v>7</v>
       </c>
       <c r="U173">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V173">
         <v>7</v>
@@ -12671,7 +12671,7 @@
         <v>7</v>
       </c>
       <c r="U174">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V174">
         <v>7</v>
@@ -12736,7 +12736,7 @@
         <v>7</v>
       </c>
       <c r="U175">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="V175">
         <v>7</v>
@@ -12795,7 +12795,7 @@
         <v>1</v>
       </c>
       <c r="S176" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T176">
         <v>7</v>
@@ -12931,7 +12931,7 @@
         <v>7</v>
       </c>
       <c r="U178">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V178">
         <v>7</v>
@@ -12996,7 +12996,7 @@
         <v>7</v>
       </c>
       <c r="U179">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="V179">
         <v>7</v>
@@ -13061,7 +13061,7 @@
         <v>7</v>
       </c>
       <c r="U180">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V180">
         <v>7</v>
@@ -13126,7 +13126,7 @@
         <v>7</v>
       </c>
       <c r="U181">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="V181">
         <v>7</v>
@@ -13256,7 +13256,7 @@
         <v>7</v>
       </c>
       <c r="U183">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="V183">
         <v>7</v>
@@ -13646,7 +13646,7 @@
         <v>7</v>
       </c>
       <c r="U189">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="V189">
         <v>7</v>
@@ -13926,7 +13926,7 @@
         <v>25</v>
       </c>
       <c r="D194" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E194">
         <v>7</v>
@@ -13962,7 +13962,7 @@
         <v>1</v>
       </c>
       <c r="R194" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S194" t="b">
         <v>1</v>
@@ -14056,7 +14056,7 @@
         <v>25</v>
       </c>
       <c r="D196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E196">
         <v>7</v>
@@ -14092,7 +14092,7 @@
         <v>1</v>
       </c>
       <c r="R196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S196" t="b">
         <v>1</v>
@@ -14101,7 +14101,7 @@
         <v>6</v>
       </c>
       <c r="U196">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="V196">
         <v>6</v>
@@ -14296,7 +14296,7 @@
         <v>7</v>
       </c>
       <c r="U199">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="V199">
         <v>7</v>
@@ -14361,7 +14361,7 @@
         <v>7</v>
       </c>
       <c r="U200">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="V200">
         <v>7</v>
@@ -14491,7 +14491,7 @@
         <v>7</v>
       </c>
       <c r="U202">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V202">
         <v>7</v>
@@ -14511,7 +14511,7 @@
         <v>25</v>
       </c>
       <c r="D203" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E203">
         <v>7</v>
@@ -14550,13 +14550,13 @@
         <v>1</v>
       </c>
       <c r="S203" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T203">
         <v>7</v>
       </c>
       <c r="U203">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="V203">
         <v>7</v>
@@ -14881,7 +14881,7 @@
         <v>7</v>
       </c>
       <c r="U208">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V208">
         <v>7</v>
@@ -15200,7 +15200,7 @@
         <v>1</v>
       </c>
       <c r="S213" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T213">
         <v>7</v>
@@ -15265,7 +15265,7 @@
         <v>0</v>
       </c>
       <c r="S214" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T214">
         <v>5</v>
@@ -15590,7 +15590,7 @@
         <v>1</v>
       </c>
       <c r="S219" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T219">
         <v>7</v>
@@ -15791,7 +15791,7 @@
         <v>7</v>
       </c>
       <c r="U222">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="V222">
         <v>7</v>
@@ -15856,7 +15856,7 @@
         <v>7</v>
       </c>
       <c r="U223">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="V223">
         <v>7</v>
@@ -15980,7 +15980,7 @@
         <v>1</v>
       </c>
       <c r="S225" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T225">
         <v>7</v>
@@ -16181,7 +16181,7 @@
         <v>7</v>
       </c>
       <c r="U228">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="V228">
         <v>7</v>
@@ -16266,7 +16266,7 @@
         <v>26</v>
       </c>
       <c r="D230" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E230">
         <v>7</v>
@@ -16305,13 +16305,13 @@
         <v>1</v>
       </c>
       <c r="S230" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T230">
         <v>7</v>
       </c>
       <c r="U230">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="V230">
         <v>7</v>
@@ -16435,7 +16435,7 @@
         <v>1</v>
       </c>
       <c r="S232" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T232">
         <v>7</v>
@@ -16636,7 +16636,7 @@
         <v>7</v>
       </c>
       <c r="U235">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="V235">
         <v>7</v>
@@ -16721,7 +16721,7 @@
         <v>27</v>
       </c>
       <c r="D237" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E237">
         <v>7</v>
@@ -16757,7 +16757,7 @@
         <v>1</v>
       </c>
       <c r="R237" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S237" t="b">
         <v>1</v>
@@ -16766,7 +16766,7 @@
         <v>6</v>
       </c>
       <c r="U237">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="V237">
         <v>6</v>
@@ -16786,7 +16786,7 @@
         <v>27</v>
       </c>
       <c r="D238" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E238">
         <v>7</v>
@@ -16822,7 +16822,7 @@
         <v>1</v>
       </c>
       <c r="R238" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S238" t="b">
         <v>1</v>
@@ -16831,7 +16831,7 @@
         <v>7</v>
       </c>
       <c r="U238">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="V238">
         <v>7</v>
@@ -16851,7 +16851,7 @@
         <v>27</v>
       </c>
       <c r="D239" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E239">
         <v>7</v>
@@ -16887,7 +16887,7 @@
         <v>1</v>
       </c>
       <c r="R239" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S239" t="b">
         <v>1</v>
@@ -16896,7 +16896,7 @@
         <v>7</v>
       </c>
       <c r="U239">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="V239">
         <v>7</v>
@@ -16916,7 +16916,7 @@
         <v>27</v>
       </c>
       <c r="D240" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E240">
         <v>7</v>
@@ -16952,7 +16952,7 @@
         <v>1</v>
       </c>
       <c r="R240" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S240" t="b">
         <v>1</v>
@@ -16961,7 +16961,7 @@
         <v>6</v>
       </c>
       <c r="U240">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="V240">
         <v>6</v>
@@ -17017,7 +17017,7 @@
         <v>0</v>
       </c>
       <c r="R241" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S241" t="b">
         <v>0</v>
@@ -17147,10 +17147,10 @@
         <v>0</v>
       </c>
       <c r="R243" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S243" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T243">
         <v>7</v>
@@ -17306,7 +17306,7 @@
         <v>27</v>
       </c>
       <c r="D246" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E246">
         <v>7</v>
@@ -17342,7 +17342,7 @@
         <v>1</v>
       </c>
       <c r="R246" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S246" t="b">
         <v>1</v>
@@ -17351,7 +17351,7 @@
         <v>7</v>
       </c>
       <c r="U246">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="V246">
         <v>7</v>
@@ -17472,10 +17472,10 @@
         <v>0</v>
       </c>
       <c r="R248" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S248" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T248">
         <v>7</v>
@@ -17501,7 +17501,7 @@
         <v>27</v>
       </c>
       <c r="D249" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E249">
         <v>7</v>
@@ -17537,7 +17537,7 @@
         <v>1</v>
       </c>
       <c r="R249" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S249" t="b">
         <v>1</v>
@@ -17546,7 +17546,7 @@
         <v>6</v>
       </c>
       <c r="U249">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="V249">
         <v>6</v>
@@ -17605,7 +17605,7 @@
         <v>0</v>
       </c>
       <c r="S250" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T250">
         <v>3</v>
@@ -17667,10 +17667,10 @@
         <v>0</v>
       </c>
       <c r="R251" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S251" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T251">
         <v>7</v>
@@ -17806,7 +17806,7 @@
         <v>7</v>
       </c>
       <c r="U253">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="V253">
         <v>7</v>
@@ -17865,7 +17865,7 @@
         <v>0</v>
       </c>
       <c r="S254" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T254">
         <v>4</v>
@@ -18001,7 +18001,7 @@
         <v>7</v>
       </c>
       <c r="U256">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="V256">
         <v>7</v>
@@ -18066,7 +18066,7 @@
         <v>7</v>
       </c>
       <c r="U257">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="V257">
         <v>7</v>
@@ -18131,7 +18131,7 @@
         <v>7</v>
       </c>
       <c r="U258">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="V258">
         <v>7</v>
@@ -18456,7 +18456,7 @@
         <v>7</v>
       </c>
       <c r="U263">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="V263">
         <v>7</v>
@@ -18521,7 +18521,7 @@
         <v>7</v>
       </c>
       <c r="U264">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V264">
         <v>7</v>
@@ -18846,7 +18846,7 @@
         <v>7</v>
       </c>
       <c r="U269">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V269">
         <v>7</v>
@@ -18866,7 +18866,7 @@
         <v>28</v>
       </c>
       <c r="D270" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E270">
         <v>7</v>
@@ -18905,13 +18905,13 @@
         <v>1</v>
       </c>
       <c r="S270" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T270">
         <v>7</v>
       </c>
       <c r="U270">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="V270">
         <v>7</v>
@@ -19041,7 +19041,7 @@
         <v>7</v>
       </c>
       <c r="U272">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V272">
         <v>7</v>
@@ -19171,7 +19171,7 @@
         <v>7</v>
       </c>
       <c r="U274">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="V274">
         <v>7</v>
@@ -19236,7 +19236,7 @@
         <v>7</v>
       </c>
       <c r="U275">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="V275">
         <v>7</v>
@@ -19295,7 +19295,7 @@
         <v>1</v>
       </c>
       <c r="S276" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T276">
         <v>7</v>
@@ -19561,7 +19561,7 @@
         <v>7</v>
       </c>
       <c r="U280">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="V280">
         <v>7</v>
@@ -19646,7 +19646,7 @@
         <v>28</v>
       </c>
       <c r="D282" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E282">
         <v>7</v>
@@ -19685,13 +19685,13 @@
         <v>1</v>
       </c>
       <c r="S282" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T282">
         <v>7</v>
       </c>
       <c r="U282">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="V282">
         <v>7</v>
@@ -19756,7 +19756,7 @@
         <v>7</v>
       </c>
       <c r="U283">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V283">
         <v>7</v>
@@ -19821,7 +19821,7 @@
         <v>6</v>
       </c>
       <c r="U284">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="V284">
         <v>6</v>
@@ -19886,7 +19886,7 @@
         <v>7</v>
       </c>
       <c r="U285">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="V285">
         <v>7</v>
@@ -20276,7 +20276,7 @@
         <v>7</v>
       </c>
       <c r="U291">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V291">
         <v>7</v>

</xml_diff>

<commit_message>
modificando nombre logueo interno
</commit_message>
<xml_diff>
--- a/codigo/datasets/datasets_aumentados/logs/pcsmote/por_muestras/log_pcsmote_x_muestra_ecoli.xlsx
+++ b/codigo/datasets/datasets_aumentados/logs/pcsmote/por_muestras/log_pcsmote_x_muestra_ecoli.xlsx
@@ -88,10 +88,10 @@
     <t>cant_min_en_p_elegido</t>
   </si>
   <si>
-    <t>D35_R35_Pentropia</t>
+    <t>PRD35_PR35_CPent_UD080_PE45</t>
   </si>
   <si>
-    <t>D35_R35_Pproporcion</t>
+    <t>PRD35_PR35_CPprop_UD080_Ppp041</t>
   </si>
   <si>
     <t>im</t>

</xml_diff>